<commit_message>
docs(platform): 설계서 V3 갱신 — NBA 언급 제거 + JWT secret 위치 정합
- NBA(next_best_action) 언급 4곳 자연스럽게 제거 (행/흐름은 유지)
- JWT secret 위치 4곳 SSM /lifesync360/jwt-secret -> Secrets Manager ecs-jwt-signing
  (실 운영 변경 반영: afe34df fix(security) 후 cda776b 시점에 이전 완료)
- build_platform_xlsx.py OUT 경로 상대경로화 (다른 환경에서도 동작)
- xlsx 재생성
</commit_message>
<xml_diff>
--- a/lifesync360-platform 설계서 V3.xlsx
+++ b/lifesync360-platform 설계서 V3.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="인증 · 로그인" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="홈 · 점수 · 캠페인" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="추천 · 상품" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="이벤트 · 신청 내역" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="동의 · 설정" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="인프라 · 운영" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="인증 · 로그인" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="홈 · 점수 · 캠페인" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="추천 · 상품" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="이벤트 · 신청 내역" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="동의 · 설정" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="인프라 · 운영" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -572,12 +572,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>AWS Systems Manager (Parameter Store)</t>
+          <t>AWS Secrets Manager</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>/lifesync360/jwt-secret (SecureString)</t>
+          <t>ecs-jwt-signing · jwt key</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -599,17 +599,17 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>AWS Systems Manager (Parameter Store)</t>
+          <t>AWS Secrets Manager</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>/lifesync360/jwt-secret (SecureString)</t>
+          <t>ecs-jwt-signing · jwt key</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>첫 호출 1회만 SSM 조회 후 메모리 캐시. ECS 배포 시 환경변수로 자동 주입</t>
+          <t>첫 호출 1회만 Secrets Manager 조회 후 메모리 캐시. ECS 배포 시 환경변수로 자동 주입</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>입력: 이메일·비밀번호 / 검증: test_login_credentials.csv (5 등급 데모) / 토큰 발급: jwt.encode + SSM /lifesync360/jwt-secret</t>
+          <t>입력: 이메일·비밀번호 / 검증: test_login_credentials.csv (5 등급 데모) / 토큰 발급: jwt.encode + Secrets Manager ecs-jwt-signing</t>
         </is>
       </c>
     </row>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>추천 정렬에 필요한 본인 점수·등급·NBA 가져오기</t>
+          <t>추천 정렬에 필요한 본인 점수·등급 가져오기</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>등급·종합점수·건강점수·VIP 확률·다음 행동(NBA, 내부 사용)</t>
+          <t>등급·종합점수·건강점수·VIP 확률</t>
         </is>
       </c>
     </row>
@@ -1450,7 +1450,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>NBA 매칭되는 룰을 최상단으로 정렬 (내부 가중치)</t>
+          <t>등급·점수·건강조건 기준으로 우선순위 정렬</t>
         </is>
       </c>
     </row>
@@ -2618,17 +2618,17 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>AWS Systems Manager</t>
+          <t>AWS Secrets Manager</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>/lifesync360/jwt-secret</t>
+          <t>ecs-jwt-signing</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>SecureString — ECS task secrets 로 자동 주입</t>
+          <t>JSON 의 jwt key — ECS task secrets 로 자동 주입</t>
         </is>
       </c>
     </row>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>점수·등급·NBA 등 ML 산출물 저장 테이블</t>
+          <t>점수·등급 등 ML 산출물 저장 테이블</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">

</xml_diff>